<commit_message>
removed electricity from hydrogen inventories
</commit_message>
<xml_diff>
--- a/Results/Ammonia/ammonia climate change image breakdown results.xlsx
+++ b/Results/Ammonia/ammonia climate change image breakdown results.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,55 +454,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>tap water production, conventional treatment</t>
+          <t>heat production, natural gas, at industrial furnace &gt;100kW</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>market for water, deionised</t>
+          <t>market group for electricity, high voltage</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>market for nickel, class 1</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>market for tap water</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>market for solvent, organic</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>market for chemical factory, organics</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>catalysts for ammonia synthesis from SMR</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>carbon dioxide MEA capture, without energy consumption and flue gas emissions</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>activated carbon production, granular from hard coal</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>natural gas burnt in furnace excluding carbon dioxide generated in flue gas</t>
+          <t>market for municipal solid waste</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>market group for electricity, high voltage</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>treatment of inert waste, inert material landfill</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>treatment of wastewater, average, capacity 1E9l/year</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>direct emissions</t>
         </is>
@@ -523,43 +508,34 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2.412940089071636</v>
+        <v>2.70138576098771</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2140792972850464</v>
+        <v>0.1781930729128459</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0003470375133943524</v>
+        <v>0.9912794650313742</v>
       </c>
       <c r="G2" t="n">
-        <v>4.668693119096242e-06</v>
+        <v>0.03460102011223961</v>
       </c>
       <c r="H2" t="n">
-        <v>0.05667744160421465</v>
+        <v>0.007206185811343898</v>
       </c>
       <c r="I2" t="n">
-        <v>0.001321100887615479</v>
+        <v>0.0008618266545860042</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01167314207452211</v>
+        <v>2.371044458602718e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.0007333049244907387</v>
+        <v>0.05638557894879985</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002349112560517623</v>
       </c>
       <c r="M2" t="n">
-        <v>0.6571326333470894</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1.698161765630896e-06</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.0001159612641747771</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1.467340447171525</v>
+        <v>1.432599989815883</v>
       </c>
     </row>
     <row r="3">
@@ -577,43 +553,34 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.380092676391155</v>
+        <v>2.691875379548547</v>
       </c>
       <c r="E3" t="n">
-        <v>0.212466587729354</v>
+        <v>0.1768507027019514</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0003330462605220726</v>
+        <v>0.9886740998015557</v>
       </c>
       <c r="G3" t="n">
-        <v>4.491717305687886e-06</v>
+        <v>0.03317665334590966</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05273875905007323</v>
+        <v>0.007026354226836978</v>
       </c>
       <c r="I3" t="n">
-        <v>0.001278716966860691</v>
+        <v>0.0008225847373114109</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01148112202478894</v>
+        <v>2.301798502710315e-05</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.0007259840405397901</v>
+        <v>0.05246717879126209</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002347979558317269</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6300814689312937</v>
-      </c>
-      <c r="N3" t="n">
-        <v>1.578917436305303e-06</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.0001124757378675934</v>
-      </c>
-      <c r="P3" t="n">
-        <v>1.467340447102533</v>
+        <v>1.432599990002861</v>
       </c>
     </row>
     <row r="4">
@@ -631,43 +598,34 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.364475380583007</v>
+        <v>2.687453749981444</v>
       </c>
       <c r="E4" t="n">
-        <v>0.211226769572796</v>
+        <v>0.1758187159102714</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0003251818982956253</v>
+        <v>0.9869208102975424</v>
       </c>
       <c r="G4" t="n">
-        <v>4.398738613997763e-06</v>
+        <v>0.03245623250075627</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05207212567319383</v>
+        <v>0.00680261990627155</v>
       </c>
       <c r="I4" t="n">
-        <v>0.001254373518574717</v>
+        <v>0.0007942733092764942</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01148353747448077</v>
+        <v>2.253727091543773e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.0007215106498854025</v>
+        <v>0.05180397826847868</v>
       </c>
       <c r="L4" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002345924114672454</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6163994432118748</v>
-      </c>
-      <c r="N4" t="n">
-        <v>1.366382463432784e-06</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.0001092816753008211</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1.467340447093639</v>
+        <v>1.432599990106465</v>
       </c>
     </row>
     <row r="5">
@@ -685,43 +643,34 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.322245248700793</v>
+        <v>2.682707270890122</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2099956643250808</v>
+        <v>0.1747939814779771</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0003052647699732962</v>
+        <v>0.9846717895247182</v>
       </c>
       <c r="G5" t="n">
-        <v>4.278496916899577e-06</v>
+        <v>0.03024969660957806</v>
       </c>
       <c r="H5" t="n">
-        <v>0.05297954861637624</v>
+        <v>0.006684167291090686</v>
       </c>
       <c r="I5" t="n">
-        <v>0.001220236614516904</v>
+        <v>0.0007440003100120236</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01153172184604976</v>
+        <v>2.241103424424512e-05</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.0007124884591590286</v>
+        <v>0.05270672840247491</v>
       </c>
       <c r="L5" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002345059905963856</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5744935474885341</v>
-      </c>
-      <c r="N5" t="n">
-        <v>1.244174819400435e-06</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.0001058178019317261</v>
-      </c>
-      <c r="P5" t="n">
-        <v>1.467340447032094</v>
+        <v>1.43259999024943</v>
       </c>
     </row>
     <row r="6">
@@ -739,43 +688,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.905967710444639</v>
+        <v>2.617363805126579</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1996592787732956</v>
+        <v>0.1661902896327437</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0001236411135047592</v>
+        <v>0.9700611888767104</v>
       </c>
       <c r="G6" t="n">
-        <v>2.832253237472474e-06</v>
+        <v>0.01005965082288591</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03222277284471087</v>
+        <v>0.005799706389261776</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0008401758747966132</v>
+        <v>0.0003419697889473611</v>
       </c>
       <c r="J6" t="n">
-        <v>0.010301282813645</v>
+        <v>1.983272969684714e-05</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.0006367033450698021</v>
+        <v>0.03205684044231071</v>
       </c>
       <c r="L6" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002343347748338776</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1910499983628199</v>
-      </c>
-      <c r="N6" t="n">
-        <v>9.950567923838702e-07</v>
-      </c>
-      <c r="O6" t="n">
-        <v>8.302458737330606e-05</v>
-      </c>
-      <c r="P6" t="n">
-        <v>1.467340446115873</v>
+        <v>1.432599991669188</v>
       </c>
     </row>
     <row r="7">
@@ -793,43 +733,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.630043710779226</v>
+        <v>2.571327769745714</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1913946435114436</v>
+        <v>0.1593110594947062</v>
       </c>
       <c r="F7" t="n">
-        <v>1.414879126306024e-06</v>
+        <v>0.9584674809095466</v>
       </c>
       <c r="G7" t="n">
-        <v>1.833967683161032e-06</v>
+        <v>-0.003285036645751893</v>
       </c>
       <c r="H7" t="n">
-        <v>0.01909226364099607</v>
+        <v>0.004930059965408335</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0005795707703121277</v>
+        <v>5.869354087820758e-05</v>
       </c>
       <c r="J7" t="n">
-        <v>0.009559567049876537</v>
+        <v>1.770885490023403e-05</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.000583768283111928</v>
+        <v>0.01899394729843688</v>
       </c>
       <c r="L7" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002338636394675151</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.06238847220868639</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4.208752861818437e-07</v>
-      </c>
-      <c r="O7" t="n">
-        <v>6.582502683039843e-05</v>
-      </c>
-      <c r="P7" t="n">
-        <v>1.46734044555581</v>
+        <v>1.432599992688122</v>
       </c>
     </row>
     <row r="8">
@@ -847,43 +778,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.577247635959622</v>
+        <v>2.560232389002389</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1891429464580232</v>
+        <v>0.1574368155939351</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.208628183159783e-05</v>
+        <v>0.9551065726301154</v>
       </c>
       <c r="G8" t="n">
-        <v>1.61650312870015e-06</v>
+        <v>-0.005772129338216924</v>
       </c>
       <c r="H8" t="n">
-        <v>0.01602111112009202</v>
+        <v>0.004673778925411242</v>
       </c>
       <c r="I8" t="n">
-        <v>0.000522736555117797</v>
+        <v>-1.962395166061771e-06</v>
       </c>
       <c r="J8" t="n">
-        <v>0.009394983654022148</v>
+        <v>1.704250781520692e-05</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.0005732155089807655</v>
+        <v>0.01593860979501701</v>
       </c>
       <c r="L8" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002336683504582249</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.1096226221001142</v>
-      </c>
-      <c r="N8" t="n">
-        <v>1.430493603757126e-07</v>
-      </c>
-      <c r="O8" t="n">
-        <v>6.161105308375183e-05</v>
-      </c>
-      <c r="P8" t="n">
-        <v>1.467340445464061</v>
+        <v>1.43259999293302</v>
       </c>
     </row>
     <row r="9">
@@ -901,43 +823,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.262949382451287</v>
+        <v>2.67190713848965</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2088904102326467</v>
+        <v>0.1738740017060979</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0002813573641260573</v>
+        <v>0.9832687071252696</v>
       </c>
       <c r="G9" t="n">
-        <v>4.059071515519766e-06</v>
+        <v>0.02750481817620907</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04734035821922424</v>
+        <v>0.006609265309916262</v>
       </c>
       <c r="I9" t="n">
-        <v>0.001160619215876863</v>
+        <v>0.0006969252099904687</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01118696502873083</v>
+        <v>2.220253166416692e-05</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.0007038213519493984</v>
+        <v>0.0470965772321671</v>
       </c>
       <c r="L9" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002346507511055393</v>
       </c>
       <c r="M9" t="n">
-        <v>0.52236360486585</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1.396637554217418e-06</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.000104020306094437</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1.467340446867957</v>
+        <v>1.43259999044723</v>
       </c>
     </row>
     <row r="10">
@@ -955,43 +868,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.884004147060415</v>
+        <v>2.613204401487478</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1988653112809577</v>
+        <v>0.1655294153256679</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0001139009061973322</v>
+        <v>0.9689336783023136</v>
       </c>
       <c r="G10" t="n">
-        <v>2.740618887869465e-06</v>
+        <v>0.009014879625393841</v>
       </c>
       <c r="H10" t="n">
-        <v>0.03098602110776474</v>
+        <v>0.005729824681282371</v>
       </c>
       <c r="I10" t="n">
-        <v>0.000815249528333088</v>
+        <v>0.0003162743532320328</v>
       </c>
       <c r="J10" t="n">
-        <v>0.01024386407335333</v>
+        <v>1.965874688772684e-05</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.0006336232016978827</v>
+        <v>0.03082645740578252</v>
       </c>
       <c r="L10" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.000234221286308663</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1712080039353114</v>
-      </c>
-      <c r="N10" t="n">
-        <v>8.871887447016927e-07</v>
-      </c>
-      <c r="O10" t="n">
-        <v>8.137955552979872e-05</v>
-      </c>
-      <c r="P10" t="n">
-        <v>1.467340446073373</v>
+        <v>1.43259999176061</v>
       </c>
     </row>
     <row r="11">
@@ -1009,43 +913,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.650639128318577</v>
+        <v>2.578508735523657</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1928387209172635</v>
+        <v>0.1605130654510519</v>
       </c>
       <c r="F11" t="n">
-        <v>1.065162381827237e-05</v>
+        <v>0.9612120166677608</v>
       </c>
       <c r="G11" t="n">
-        <v>1.946351496730475e-06</v>
+        <v>-0.002396462958093465</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02122851187051691</v>
+        <v>0.00512528270061919</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0006098192545158721</v>
+        <v>8.336780575572645e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>0.009662082753369137</v>
+        <v>1.827470994468065e-05</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.000589098742823952</v>
+        <v>0.02111919483591444</v>
       </c>
       <c r="L11" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002340037750835027</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.04551293601351529</v>
-      </c>
-      <c r="N11" t="n">
-        <v>6.084490517617899e-07</v>
-      </c>
-      <c r="O11" t="n">
-        <v>6.84102783261667e-05</v>
-      </c>
-      <c r="P11" t="n">
-        <v>1.467340445582898</v>
+        <v>1.43259999253562</v>
       </c>
     </row>
   </sheetData>
@@ -1059,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1085,60 +980,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>tap water production, conventional treatment</t>
+          <t>natural gas heating, with CCS</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>market for water, deionised</t>
+          <t>market group for electricity, high voltage</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>market for nickel, class 1</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>market for tap water</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>market for solvent, organic</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>market for chemical factory, organics</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>catalysts for ammonia synthesis from SMR</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>carbon dioxide MEA capture, without energy consumption and flue gas emissions</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>carbon dioxide transport and injection in a geological resovoir</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>natural gas burnt in furnace excluding carbon dioxide generated in flue gas</t>
+          <t>market for municipal solid waste</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>electricity with CCS, high voltage</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>heat with CCS</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>treatment of inert waste, inert material landfill</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>treatment of wastewater, average, capacity 1E9l/year</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>direct emissions</t>
         </is>
@@ -1159,46 +1034,34 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8119975218583808</v>
+        <v>1.980054957643558</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2140792972850464</v>
+        <v>0.1781930729128459</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0003470375133943524</v>
+        <v>0.4136162264855067</v>
       </c>
       <c r="G2" t="n">
-        <v>4.668693119096242e-06</v>
+        <v>0.03460102011223961</v>
       </c>
       <c r="H2" t="n">
-        <v>0.05667744160421465</v>
+        <v>0.007206185811343898</v>
       </c>
       <c r="I2" t="n">
-        <v>0.001321100887615479</v>
+        <v>0.0008618266545860042</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01406763275647539</v>
+        <v>2.371044458602718e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0198161868385776</v>
+        <v>0.05638557894879985</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002349112560517623</v>
       </c>
       <c r="M2" t="n">
-        <v>0.4131799415840956</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.02723888315574819</v>
-      </c>
-      <c r="O2" t="n">
-        <v>1.698161765630896e-06</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.0001159612641747771</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.06016770612049394</v>
+        <v>1.288932425017598</v>
       </c>
     </row>
     <row r="3">
@@ -1216,46 +1079,34 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.7739750168027139</v>
+        <v>1.963363919298775</v>
       </c>
       <c r="E3" t="n">
-        <v>0.212466587729354</v>
+        <v>0.1768507027019514</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0003330462605220726</v>
+        <v>0.4038302041772954</v>
       </c>
       <c r="G3" t="n">
-        <v>4.491717305687886e-06</v>
+        <v>0.03317665334590966</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05273875905007323</v>
+        <v>0.007026354226836978</v>
       </c>
       <c r="I3" t="n">
-        <v>0.001278716966860691</v>
+        <v>0.0008225847373114109</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01383622397859179</v>
+        <v>2.301798502710315e-05</v>
       </c>
       <c r="K3" t="n">
-        <v>0.01898362058394505</v>
+        <v>0.05246717879126209</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002347979558317269</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3824079084846204</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.02666393615674648</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1.578917436305303e-06</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.0001124757378675934</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.06016770522573078</v>
+        <v>1.288932425377349</v>
       </c>
     </row>
     <row r="4">
@@ -1273,46 +1124,34 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.755318795716069</v>
+        <v>1.955416864035832</v>
       </c>
       <c r="E4" t="n">
-        <v>0.211226769572796</v>
+        <v>0.1758187159102714</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0003251818982956253</v>
+        <v>0.3985514888926226</v>
       </c>
       <c r="G4" t="n">
-        <v>4.398738613997763e-06</v>
+        <v>0.03245623250075627</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05207212567319383</v>
+        <v>0.00680261990627155</v>
       </c>
       <c r="I4" t="n">
-        <v>0.001254373518574717</v>
+        <v>0.0007942733092764942</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01383913490514353</v>
+        <v>2.253727091543773e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>0.01827740421866645</v>
+        <v>0.05180397826847868</v>
       </c>
       <c r="L4" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002345924114672454</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3667343759984911</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.02632671233778421</v>
-      </c>
-      <c r="O4" t="n">
-        <v>1.366382463432784e-06</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.0001092816753008211</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.06016770480308564</v>
+        <v>1.288932425565772</v>
       </c>
     </row>
     <row r="5">
@@ -1330,46 +1169,34 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7059372484538927</v>
+        <v>1.938457941471321</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2099956643250808</v>
+        <v>0.1747939814779771</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0003052647699732962</v>
+        <v>0.3840900243527682</v>
       </c>
       <c r="G5" t="n">
-        <v>4.278496916899577e-06</v>
+        <v>0.03024969660957806</v>
       </c>
       <c r="H5" t="n">
-        <v>0.05297954861637624</v>
+        <v>0.006684167291090686</v>
       </c>
       <c r="I5" t="n">
-        <v>0.001220236614516904</v>
+        <v>0.0007440003100120236</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01389720325036767</v>
+        <v>2.241103424424512e-05</v>
       </c>
       <c r="K5" t="n">
-        <v>0.01716914597031695</v>
+        <v>0.05270672840247491</v>
       </c>
       <c r="L5" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002345059905963856</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3194885310522161</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.02562264391265938</v>
-      </c>
-      <c r="O5" t="n">
-        <v>1.244174819400435e-06</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.0001058178019317261</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.06016770347505762</v>
+        <v>1.288932426002579</v>
       </c>
     </row>
     <row r="6">
@@ -1387,46 +1214,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.2269215138830993</v>
+        <v>1.758255749172082</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1996592787732956</v>
+        <v>0.1661902896327437</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0001236411135047592</v>
+        <v>0.2546206944054956</v>
       </c>
       <c r="G6" t="n">
-        <v>2.832253237472474e-06</v>
+        <v>0.01005965082288591</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03222277284471087</v>
+        <v>0.005799706389261776</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0008401758747966132</v>
+        <v>0.0003419697889473611</v>
       </c>
       <c r="J6" t="n">
-        <v>0.01241436646772604</v>
+        <v>1.983272969684714e-05</v>
       </c>
       <c r="K6" t="n">
-        <v>0.008832512486519622</v>
+        <v>0.03205684044231071</v>
       </c>
       <c r="L6" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002343347748338776</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.1121016253174169</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.0196958828090798</v>
-      </c>
-      <c r="O6" t="n">
-        <v>9.950567923838702e-07</v>
-      </c>
-      <c r="P6" t="n">
-        <v>8.302458737330606e-05</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.06016769093982</v>
+        <v>1.288932430185906</v>
       </c>
     </row>
     <row r="7">
@@ -1444,46 +1259,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-0.09199690775750866</v>
+        <v>1.637631685197211</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1913946435114436</v>
+        <v>0.1593110594947062</v>
       </c>
       <c r="F7" t="n">
-        <v>1.414879126306024e-06</v>
+        <v>0.1684389560496941</v>
       </c>
       <c r="G7" t="n">
-        <v>1.833967683161032e-06</v>
+        <v>-0.003285036645751893</v>
       </c>
       <c r="H7" t="n">
-        <v>0.01909226364099607</v>
+        <v>0.004930059965408335</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0005795707703121277</v>
+        <v>5.869354087820758e-05</v>
       </c>
       <c r="J7" t="n">
-        <v>0.01152050388062046</v>
+        <v>1.770885490023403e-05</v>
       </c>
       <c r="K7" t="n">
-        <v>0.002483476575502545</v>
+        <v>0.01899394729843688</v>
       </c>
       <c r="L7" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002338636394675151</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.3978557426339674</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.01557123305086402</v>
-      </c>
-      <c r="O7" t="n">
-        <v>4.208752861818437e-07</v>
-      </c>
-      <c r="P7" t="n">
-        <v>6.582502683039843e-05</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.06016768270413414</v>
+        <v>1.288932432999471</v>
       </c>
     </row>
     <row r="8">
@@ -1501,46 +1304,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-0.1539181285496789</v>
+        <v>1.613376427610021</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1891429464580232</v>
+        <v>0.1574368155939351</v>
       </c>
       <c r="F8" t="n">
-        <v>-2.208628183159783e-05</v>
+        <v>0.1519181706097656</v>
       </c>
       <c r="G8" t="n">
-        <v>1.61650312870015e-06</v>
+        <v>-0.005772129338216924</v>
       </c>
       <c r="H8" t="n">
-        <v>0.01602111112009202</v>
+        <v>0.004673778925411242</v>
       </c>
       <c r="I8" t="n">
-        <v>0.000522736555117797</v>
+        <v>-1.962395166061771e-06</v>
       </c>
       <c r="J8" t="n">
-        <v>0.01132215978818057</v>
+        <v>1.704250781520692e-05</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0006918155856223472</v>
+        <v>0.01593860979501701</v>
       </c>
       <c r="L8" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002336683504582249</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.4514733887796771</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.01466555922144343</v>
-      </c>
-      <c r="O8" t="n">
-        <v>1.430493603757126e-07</v>
-      </c>
-      <c r="P8" t="n">
-        <v>6.161105308375183e-05</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.06016768118411786</v>
+        <v>1.288932433561001</v>
       </c>
     </row>
     <row r="9">
@@ -1558,46 +1349,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.6384329299075047</v>
+        <v>1.911698651310101</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2088904102326467</v>
+        <v>0.1738740017060979</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0002813573641260573</v>
+        <v>0.3667277838085859</v>
       </c>
       <c r="G9" t="n">
-        <v>4.059071515519766e-06</v>
+        <v>0.02750481817620907</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04734035821922424</v>
+        <v>0.006609265309916262</v>
       </c>
       <c r="I9" t="n">
-        <v>0.001160619215876863</v>
+        <v>0.0006969252099904687</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01348172708590641</v>
+        <v>2.220253166416692e-05</v>
       </c>
       <c r="K9" t="n">
-        <v>0.01625994546029095</v>
+        <v>0.0470965772321671</v>
       </c>
       <c r="L9" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002346507511055393</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2608925934057818</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.02486877518749302</v>
-      </c>
-      <c r="O9" t="n">
-        <v>1.396637554217418e-06</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.000104020306094437</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.06016770172733477</v>
+        <v>1.288932426584364</v>
       </c>
     </row>
     <row r="10">
@@ -1615,46 +1394,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.2014383412291763</v>
+        <v>1.748387653021136</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1988653112809577</v>
+        <v>0.1655294153256679</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0001139009061973322</v>
+        <v>0.2477844911819007</v>
       </c>
       <c r="G10" t="n">
-        <v>2.740618887869465e-06</v>
+        <v>0.009014879625393841</v>
       </c>
       <c r="H10" t="n">
-        <v>0.03098602110776474</v>
+        <v>0.005729824681282371</v>
       </c>
       <c r="I10" t="n">
-        <v>0.000815249528333088</v>
+        <v>0.0003162743532320328</v>
       </c>
       <c r="J10" t="n">
-        <v>0.01234516952429762</v>
+        <v>1.965874688772684e-05</v>
       </c>
       <c r="K10" t="n">
-        <v>0.008257254349559965</v>
+        <v>0.03082645740578252</v>
       </c>
       <c r="L10" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.000234221286308663</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.1345270472525631</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.01934981813138773</v>
-      </c>
-      <c r="O10" t="n">
-        <v>8.871887447016927e-07</v>
-      </c>
-      <c r="P10" t="n">
-        <v>8.137955552979872e-05</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.06016769029641905</v>
+        <v>1.28893243041468</v>
       </c>
     </row>
     <row r="11">
@@ -1672,46 +1439,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>-0.06752947798528464</v>
+        <v>1.648261735304907</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1928387209172635</v>
+        <v>0.1605130654510519</v>
       </c>
       <c r="F11" t="n">
-        <v>1.065162381827237e-05</v>
+        <v>0.1746325762206515</v>
       </c>
       <c r="G11" t="n">
-        <v>1.946351496730475e-06</v>
+        <v>-0.002396462958093465</v>
       </c>
       <c r="H11" t="n">
-        <v>0.02122851187051691</v>
+        <v>0.00512528270061919</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0006098192545158721</v>
+        <v>8.336780575572645e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>0.01164404844636794</v>
+        <v>1.827470994468065e-05</v>
       </c>
       <c r="K11" t="n">
-        <v>0.003302009428422227</v>
+        <v>0.02111919483591444</v>
       </c>
       <c r="L11" t="n">
-        <v>0.00497996599365975</v>
+        <v>0.0002340037750835027</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.3784239351821365</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.01604208133628745</v>
-      </c>
-      <c r="O11" t="n">
-        <v>6.084490517617899e-07</v>
-      </c>
-      <c r="P11" t="n">
-        <v>6.84102783261667e-05</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.06016768324712521</v>
+        <v>1.28893243276398</v>
       </c>
     </row>
   </sheetData>
@@ -1795,28 +1550,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8720213113269694</v>
+        <v>0.8720213113269696</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003092854659228074</v>
+        <v>0.0003092854659228066</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0001294472502647097</v>
+        <v>0.0001294472502647094</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04661719571946651</v>
+        <v>0.04661719571946643</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3907655017550623</v>
+        <v>0.3907655017550621</v>
       </c>
       <c r="I2" t="n">
-        <v>2.879037331884943e-07</v>
+        <v>2.879037331885099e-07</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4257626002063724</v>
+        <v>0.4257626002063719</v>
       </c>
       <c r="K2" t="n">
-        <v>0.008436993026147532</v>
+        <v>0.008436993026148421</v>
       </c>
     </row>
     <row r="3">
@@ -1834,28 +1589,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.809885205190117</v>
+        <v>0.8098852051901169</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0002911484276349664</v>
+        <v>0.0002911484276349665</v>
       </c>
       <c r="F3" t="n">
-        <v>0.000123471618988912</v>
+        <v>0.0001234716189889123</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04337762931868518</v>
+        <v>0.0433776293186852</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3746794617388221</v>
+        <v>0.3746794617388228</v>
       </c>
       <c r="I3" t="n">
-        <v>2.676872330474532e-07</v>
+        <v>2.676872330474503e-07</v>
       </c>
       <c r="J3" t="n">
-        <v>0.382976232915369</v>
+        <v>0.3829762329153686</v>
       </c>
       <c r="K3" t="n">
-        <v>0.008436993483383781</v>
+        <v>0.008436993483383337</v>
       </c>
     </row>
     <row r="4">
@@ -1873,28 +1628,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.7651623798065252</v>
+        <v>0.7651623798065263</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0002872574103545492</v>
+        <v>0.0002872574103545495</v>
       </c>
       <c r="F4" t="n">
         <v>0.0001213610495604623</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04282932336620182</v>
+        <v>0.04282932336620195</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3665434122201091</v>
+        <v>0.3665434122201103</v>
       </c>
       <c r="I4" t="n">
-        <v>2.316543807235277e-07</v>
+        <v>2.316543807235276e-07</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3469438003334519</v>
+        <v>0.3469438003334512</v>
       </c>
       <c r="K4" t="n">
-        <v>0.00843699377246665</v>
+        <v>0.008436993772467205</v>
       </c>
     </row>
     <row r="5">
@@ -1912,28 +1667,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7342814462012456</v>
+        <v>0.7342814462012486</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0002867077540194825</v>
+        <v>0.0002867077540194822</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0001166652843311128</v>
+        <v>0.000116665284331113</v>
       </c>
       <c r="G5" t="n">
         <v>0.04357567873696951</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3416239704851606</v>
+        <v>0.3416239704851618</v>
       </c>
       <c r="I5" t="n">
-        <v>2.109354847660986e-07</v>
+        <v>2.109354847660368e-07</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3402412189539439</v>
+        <v>0.3402412189539448</v>
       </c>
       <c r="K5" t="n">
-        <v>0.008436994051336244</v>
+        <v>0.008436994051337132</v>
       </c>
     </row>
     <row r="6">
@@ -1951,28 +1706,28 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.4239314081899944</v>
+        <v>0.4239314081899941</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0001687669064447476</v>
+        <v>0.0001687669064447477</v>
       </c>
       <c r="F6" t="n">
-        <v>5.340922497879632e-05</v>
+        <v>5.340922497879639e-05</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02650323066477471</v>
+        <v>0.02650323066477468</v>
       </c>
       <c r="H6" t="n">
         <v>0.1136083412724361</v>
       </c>
       <c r="I6" t="n">
-        <v>1.687003977241576e-07</v>
+        <v>1.687003977241577e-07</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2751604943556245</v>
+        <v>0.2751604943556225</v>
       </c>
       <c r="K6" t="n">
-        <v>0.008436997065337848</v>
+        <v>0.008436997065339569</v>
       </c>
     </row>
     <row r="7">
@@ -1990,28 +1745,28 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.1831150589446081</v>
+        <v>0.1831150589446079</v>
       </c>
       <c r="E7" t="n">
-        <v>9.409785458113981e-05</v>
+        <v>9.409785458114016e-05</v>
       </c>
       <c r="F7" t="n">
-        <v>1.186428933566405e-05</v>
+        <v>1.186428933566429e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.01570338684471925</v>
+        <v>0.01570338684471926</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0370994551315823</v>
+        <v>-0.03709945513158227</v>
       </c>
       <c r="I7" t="n">
         <v>7.135454851882994e-08</v>
       </c>
       <c r="J7" t="n">
-        <v>0.195968094488482</v>
+        <v>0.1959680944884817</v>
       </c>
       <c r="K7" t="n">
-        <v>0.008436999244523791</v>
+        <v>0.008436999244523846</v>
       </c>
     </row>
     <row r="8">
@@ -2029,28 +1784,28 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.1339261033626204</v>
+        <v>0.1339261033626203</v>
       </c>
       <c r="E8" t="n">
-        <v>7.858333797517887e-05</v>
+        <v>7.858333797517846e-05</v>
       </c>
       <c r="F8" t="n">
-        <v>3.625526732741283e-06</v>
+        <v>3.625526732741113e-06</v>
       </c>
       <c r="G8" t="n">
-        <v>0.01317736389627568</v>
+        <v>0.01317736389627566</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.06518735602958656</v>
+        <v>-0.06518735602958659</v>
       </c>
       <c r="I8" t="n">
-        <v>2.425236848218572e-08</v>
+        <v>2.425236848215814e-08</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1774168626981575</v>
+        <v>0.177416862698158</v>
       </c>
       <c r="K8" t="n">
-        <v>0.008436999680697388</v>
+        <v>0.008436999680696805</v>
       </c>
     </row>
     <row r="9">
@@ -2068,28 +1823,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.7078565218301056</v>
+        <v>0.7078565218301038</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0002595616031116234</v>
+        <v>0.0002595616031116237</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0001061573509949633</v>
+        <v>0.000106157350994963</v>
       </c>
       <c r="G9" t="n">
-        <v>0.03893744463531202</v>
+        <v>0.03893744463531196</v>
       </c>
       <c r="H9" t="n">
-        <v>0.310624774658196</v>
+        <v>0.3106247746581955</v>
       </c>
       <c r="I9" t="n">
-        <v>2.367837822688315e-07</v>
+        <v>2.367837822688863e-07</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3494913523928275</v>
+        <v>0.349491352392827</v>
       </c>
       <c r="K9" t="n">
-        <v>0.008436994405881304</v>
+        <v>0.008436994405880638</v>
       </c>
     </row>
     <row r="10">
@@ -2107,28 +1862,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.3904687354326865</v>
+        <v>0.3904687354326883</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0001622073495586278</v>
+        <v>0.0001622073495586281</v>
       </c>
       <c r="F10" t="n">
-        <v>5.004137427753086e-05</v>
+        <v>5.004137427753117e-05</v>
       </c>
       <c r="G10" t="n">
-        <v>0.02548600236113658</v>
+        <v>0.02548600236113643</v>
       </c>
       <c r="H10" t="n">
-        <v>0.101809251538003</v>
+        <v>0.1018092515380036</v>
       </c>
       <c r="I10" t="n">
-        <v>1.504126148709638e-07</v>
+        <v>1.504126148709639e-07</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2545240850797451</v>
+        <v>0.2545240850797457</v>
       </c>
       <c r="K10" t="n">
-        <v>0.008436997317350758</v>
+        <v>0.008436997317351591</v>
       </c>
     </row>
     <row r="11">
@@ -2146,28 +1901,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.2098774376097499</v>
+        <v>0.2098774376097486</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0001031803815114755</v>
+        <v>0.0001031803815114756</v>
       </c>
       <c r="F11" t="n">
-        <v>1.556916678223189e-05</v>
+        <v>1.55691667822316e-05</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01746045101350015</v>
+        <v>0.01746045101349999</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.02706437692354484</v>
+        <v>-0.0270643769235454</v>
       </c>
       <c r="I11" t="n">
-        <v>1.031555161602287e-07</v>
+        <v>1.031555161602309e-07</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2109255117882289</v>
+        <v>0.2109255117882296</v>
       </c>
       <c r="K11" t="n">
-        <v>0.008436999027755826</v>
+        <v>0.008436999027754605</v>
       </c>
     </row>
   </sheetData>
@@ -2251,28 +2006,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.158934965895113</v>
+        <v>1.158934965895111</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003092854659228074</v>
+        <v>0.0003092854659228066</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0001294472502647097</v>
+        <v>0.0001294472502647094</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04661719571946651</v>
+        <v>0.04661719571946643</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3907655017550623</v>
+        <v>0.3907655017550621</v>
       </c>
       <c r="I2" t="n">
-        <v>2.879037331884943e-07</v>
+        <v>2.879037331885099e-07</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7126762563291841</v>
+        <v>0.7126762563291845</v>
       </c>
       <c r="K2" t="n">
-        <v>0.008436991471479471</v>
+        <v>0.008436991471477251</v>
       </c>
     </row>
     <row r="3">
@@ -2293,25 +2048,25 @@
         <v>1.021863442698996</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0002911484276349664</v>
+        <v>0.0002911484276349665</v>
       </c>
       <c r="F3" t="n">
-        <v>0.000123471618988912</v>
+        <v>0.0001234716189889123</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04337762931868518</v>
+        <v>0.0433776293186852</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3746794617388221</v>
+        <v>0.3746794617388228</v>
       </c>
       <c r="I3" t="n">
-        <v>2.676872330474532e-07</v>
+        <v>2.676872330474503e-07</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5949544715728741</v>
+        <v>0.5949544715728748</v>
       </c>
       <c r="K3" t="n">
-        <v>0.008436992334757365</v>
+        <v>0.008436992334756033</v>
       </c>
     </row>
     <row r="4">
@@ -2329,28 +2084,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.9380571426660556</v>
+        <v>0.9380571426660567</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0002872574103545492</v>
+        <v>0.0002872574103545495</v>
       </c>
       <c r="F4" t="n">
         <v>0.0001213610495604623</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04282932336620182</v>
+        <v>0.04282932336620195</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3665434122201091</v>
+        <v>0.3665434122201103</v>
       </c>
       <c r="I4" t="n">
-        <v>2.316543807235277e-07</v>
+        <v>2.316543807235276e-07</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5198385641298314</v>
+        <v>0.5198385641298313</v>
       </c>
       <c r="K4" t="n">
-        <v>0.008436992835617496</v>
+        <v>0.008436992835617385</v>
       </c>
     </row>
     <row r="5">
@@ -2371,25 +2126,25 @@
         <v>0.8873538134220893</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0002867077540194825</v>
+        <v>0.0002867077540194822</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0001166652843311128</v>
+        <v>0.000116665284331113</v>
       </c>
       <c r="G5" t="n">
         <v>0.04357567873696951</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3416239704851606</v>
+        <v>0.3416239704851618</v>
       </c>
       <c r="I5" t="n">
-        <v>2.109354847660986e-07</v>
+        <v>2.109354847660368e-07</v>
       </c>
       <c r="J5" t="n">
-        <v>0.4933135870042256</v>
+        <v>0.4933135870042252</v>
       </c>
       <c r="K5" t="n">
-        <v>0.00843699322189817</v>
+        <v>0.008436993221897504</v>
       </c>
     </row>
     <row r="6">
@@ -2407,28 +2162,28 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.5624066976108004</v>
+        <v>0.5624066976107985</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0001687669064447476</v>
+        <v>0.0001687669064447477</v>
       </c>
       <c r="F6" t="n">
-        <v>5.340922497879632e-05</v>
+        <v>5.340922497879639e-05</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02650323066477471</v>
+        <v>0.02650323066477468</v>
       </c>
       <c r="H6" t="n">
         <v>0.1136083412724361</v>
       </c>
       <c r="I6" t="n">
-        <v>1.687003977241576e-07</v>
+        <v>1.687003977241577e-07</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4136357845267695</v>
+        <v>0.4136357845267697</v>
       </c>
       <c r="K6" t="n">
-        <v>0.008436996314998835</v>
+        <v>0.008436996314996836</v>
       </c>
     </row>
     <row r="7">
@@ -2446,28 +2201,28 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.2622886342832159</v>
+        <v>0.2622886342832179</v>
       </c>
       <c r="E7" t="n">
-        <v>9.409785458113981e-05</v>
+        <v>9.409785458114016e-05</v>
       </c>
       <c r="F7" t="n">
-        <v>1.186428933566405e-05</v>
+        <v>1.186428933566429e-05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.01570338684471925</v>
+        <v>0.01570338684471926</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0370994551315823</v>
+        <v>-0.03709945513158227</v>
       </c>
       <c r="I7" t="n">
         <v>7.135454851882994e-08</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2751416702561011</v>
+        <v>0.2751416702561013</v>
       </c>
       <c r="K7" t="n">
-        <v>0.00843699881551252</v>
+        <v>0.008436998815514296</v>
       </c>
     </row>
     <row r="8">
@@ -2485,28 +2240,28 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.2025177384472989</v>
+        <v>0.2025177384472979</v>
       </c>
       <c r="E8" t="n">
-        <v>7.858333797517887e-05</v>
+        <v>7.858333797517846e-05</v>
       </c>
       <c r="F8" t="n">
-        <v>3.625526732741283e-06</v>
+        <v>3.625526732741113e-06</v>
       </c>
       <c r="G8" t="n">
-        <v>0.01317736389627568</v>
+        <v>0.01317736389627566</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.06518735602958656</v>
+        <v>-0.06518735602958659</v>
       </c>
       <c r="I8" t="n">
-        <v>2.425236848218572e-08</v>
+        <v>2.425236848215814e-08</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2460084981545067</v>
+        <v>0.2460084981545052</v>
       </c>
       <c r="K8" t="n">
-        <v>0.008436999309026638</v>
+        <v>0.008436999309027277</v>
       </c>
     </row>
     <row r="9">
@@ -2524,28 +2279,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.906267485438949</v>
+        <v>0.9062674854389478</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0002595616031116234</v>
+        <v>0.0002595616031116237</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0001061573509949633</v>
+        <v>0.000106157350994963</v>
       </c>
       <c r="G9" t="n">
-        <v>0.03893744463531202</v>
+        <v>0.03893744463531196</v>
       </c>
       <c r="H9" t="n">
-        <v>0.310624774658196</v>
+        <v>0.3106247746581955</v>
       </c>
       <c r="I9" t="n">
-        <v>2.367837822688315e-07</v>
+        <v>2.367837822688863e-07</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5479023170767818</v>
+        <v>0.5479023170767803</v>
       </c>
       <c r="K9" t="n">
-        <v>0.008436993330770304</v>
+        <v>0.008436993330771192</v>
       </c>
     </row>
     <row r="10">
@@ -2563,28 +2318,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.5011714259996428</v>
+        <v>0.5011714259996437</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0001622073495586278</v>
+        <v>0.0001622073495586281</v>
       </c>
       <c r="F10" t="n">
-        <v>5.004137427753086e-05</v>
+        <v>5.004137427753117e-05</v>
       </c>
       <c r="G10" t="n">
-        <v>0.02548600236113658</v>
+        <v>0.02548600236113643</v>
       </c>
       <c r="H10" t="n">
-        <v>0.101809251538003</v>
+        <v>0.1018092515380036</v>
       </c>
       <c r="I10" t="n">
-        <v>1.504126148709638e-07</v>
+        <v>1.504126148709639e-07</v>
       </c>
       <c r="J10" t="n">
-        <v>0.3652267762465556</v>
+        <v>0.3652267762465569</v>
       </c>
       <c r="K10" t="n">
-        <v>0.008436996717496537</v>
+        <v>0.008436996717495759</v>
       </c>
     </row>
     <row r="11">
@@ -2602,28 +2357,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.2804071502050711</v>
+        <v>0.28040715020507</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0001031803815114755</v>
+        <v>0.0001031803815114756</v>
       </c>
       <c r="F11" t="n">
-        <v>1.556916678223189e-05</v>
+        <v>1.55691667822316e-05</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01746045101350015</v>
+        <v>0.01746045101349999</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.02706437692354484</v>
+        <v>-0.0270643769235454</v>
       </c>
       <c r="I11" t="n">
-        <v>1.031555161602287e-07</v>
+        <v>1.031555161602309e-07</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2814552247657234</v>
+        <v>0.2814552247657214</v>
       </c>
       <c r="K11" t="n">
-        <v>0.008436998645582505</v>
+        <v>0.008436998645584115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>